<commit_message>
Simplifica lista de materiais para apresentação ao cliente
Consolida de 24 para 15 itens: unifica gabinete + patch panel +
organizador + régua de tomadas em um único "Rack de parede 9U-12U
completo" (eliminando a repetição da palavra "Rack" em 6 linhas
diferentes, que estava confundindo a leitura), agrupa acessórios
miúdos de cabeamento (keystones, espelhos, conectores, patch cords,
caixas de passagem, eletroduto) em 2 kits, remove ambiguidade de
especificação (ex.: "6TB ou 2x4TB" -> escolhe 6TB como padrão, com
upgrade opcional citado à parte) e limpa a coluna Local/Ponto.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fnpdJTGdpvo55JqsFcMfC
</commit_message>
<xml_diff>
--- a/SWISS-J26-Patrick/Lista_de_Materiais_Swiss_J26.xlsx
+++ b/SWISS-J26-Patrick/Lista_de_Materiais_Swiss_J26.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="127">
   <si>
     <t xml:space="preserve">Lista de Materiais — Rede Wi-Fi, CFTV e Cabeamento Estruturado</t>
   </si>
@@ -70,103 +70,121 @@
     <t xml:space="preserve">Access Point Wi-Fi 6 indoor (teto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ex.: UniFi U6-Lite / U6-Pro, dual-band, PoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-01 — Living / Circulação</t>
+    <t xml:space="preserve">UniFi U6-Lite ou equivalente, dual-band, PoE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Living / Circulação</t>
   </si>
   <si>
     <t xml:space="preserve">un</t>
   </si>
   <si>
-    <t xml:space="preserve">Cabeamento dedicado, sem cascata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-02 — Corredor das Suítes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Access Point Wi-Fi 6 externo IP65</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ex.: UniFi U6-Mesh / U6-IW, PoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-03 — Área Gourmet / Deck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Instalar sob projeção do beiral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-04 — Garagem (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opcional — avaliar com o cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suporte/bracket de fixação para AP externo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compatível com o modelo de AP escolhido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-03 / AP-04</t>
+    <t xml:space="preserve">AP-01 — cabeamento dedicado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corredor das Suítes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AP-02 — cabeamento dedicado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access Point Wi-Fi 6 externo IP65 (com suporte de fixação)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UniFi U6-Mesh ou equivalente, PoE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área Gourmet / Deck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AP-03 — sob projeção do beiral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garagem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AP-04 — item opcional, confirmar com o cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CFTV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Câmera IP bullet varifocal 4MP PoE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lente 2,8–12mm, IR 30–40m, H.265+, IP66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros laterais (leste/oeste)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAM-03, 04, 05 e 06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Câmera IP turret/dome 4MP PoE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lente fixa 2,8mm grande angular, IR 30–40m, H.265+, IP66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantos do lote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAM-01, 02, 07 e 08 — ajustar máscara de privacidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NVR 8 canais PoE + HD 6TB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compressão H.265+, gravação por movimento, retenção ~30-45 dias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escritório</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upgrade opcional: 2x4TB em RAID1 para redundância de disco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caixa de passagem externa IP65 (câmeras/AP externo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para folga e emenda de cabo PoE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perímetro externo</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">CFTV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Câmera IP bullet varifocal 4MP PoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lente 2,8–12mm, IR 30–40m, H.265+, IP66</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAM-03/04/05/06 (muros laterais)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perímetro leste/oeste</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Câmera IP turret/dome 4MP PoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lente fixa 2,8mm grande angular, IR 30–40m, H.265+, IP66</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAM-01/02/07/08 (cantos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cantos do lote — ajustar máscara de privacidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NVR 8 canais PoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compressão H.265/H.265+, saída HDMI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rack — Escritório</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HD interno para NVR (6TB) ou 2x4TB RAID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uso 24/7 (surveillance grade)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2x4TB se optar por redundância RAID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caixa de junção/passagem externa (câmeras/AP externo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IP65, para folga e emenda de cabo PoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perímetro / áreas externas</t>
+    <t xml:space="preserve">Infraestrutura Passiva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rack de parede 9U–12U completo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabinete fechado com porta ventilada + patch panel Cat6 24 portas + organizador de cabos + régua de tomadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambiente de permanência — priorizar modelo silencioso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switch PoE+ gerenciável 24 portas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget PoE compatível com 4 APs + 8 câmeras, com suporte a VLANs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nobreak 1kVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para o rack e o roteador de borda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Circuito elétrico dedicado recomendado</t>
   </si>
   <si>
     <t xml:space="preserve">Cabeamento Estruturado</t>
@@ -178,132 +196,45 @@
     <t xml:space="preserve">Uso interno, PoE-rated</t>
   </si>
   <si>
-    <t xml:space="preserve">Backbone geral (rack no Escritório)</t>
+    <t xml:space="preserve">Backbone geral (a partir do Escritório)</t>
   </si>
   <si>
     <t xml:space="preserve">cx</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa ~198m (ver aba Memória de Cálculo) — 1 caixa cobre com folga; reavaliar se o levantamento em campo indicar distâncias maiores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keystone Jack Cat6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fêmea, para pontos de TV/AP/câmera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17 pontos + reserva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminação nos pontos de rede</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espelho/placa 4x2 com saída RJ45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Padrão compatível com o restante do projeto elétrico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 pontos de TV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caixa de passagem 4x4 embutida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para pontos de AP e câmera embutidos em parede/teto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 APs + 8 câmeras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eletroduto corrugado reforçado 3/4" — rolo 50m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Embutir em laje/contrapiso pela Circulação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backbone geral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimativa ~150m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patch cord Cat6 (0,5–1,5m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pronto, com conector RJ45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patch panel ↔ switch, switch ↔ dispositivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conector RJ45 Cat6 macho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva para testes/emendas</t>
+    <t xml:space="preserve">Estimativa ~198m (ver aba Memória de Cálculo) — 1 caixa cobre com folga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit de terminação dos pontos de rede</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 keystone jacks Cat6 + 6 espelhos/placas 4x2 c/ saída RJ45 + 20 conectores RJ45 + 20 patch cords Cat6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 pontos de rede (TVs/APs/câmeras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit de infraestrutura de passagem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 caixas de passagem 4x4 embutidas + 3 rolos (50m) de eletroduto corrugado reforçado 3/4"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backbone geral (Circulação)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serviços (opcional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instalação, configuração e comissionamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mão de obra — passagem de cabos, fixação, configuração de VLANs/SSIDs, testes</t>
   </si>
   <si>
     <t xml:space="preserve">Geral</t>
   </si>
   <si>
-    <t xml:space="preserve">Infraestrutura Passiva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rack de parede / gabinete fechado 9U–12U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Porta ventilada, modelo silencioso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escritório</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambiente de permanência — priorizar baixo ruído</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patch panel Cat6 24 portas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Organizador de cabos horizontal 1U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Switch PoE+ gerenciável 24 portas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budget PoE compatível com 4 APs + 8 câmeras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suporta VLANs (item 7 do escopo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nobreak 1kVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para rack + roteador de borda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circuito elétrico dedicado recomendado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Régua de tomadas 8 vias para rack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixação em trilho 19"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serviços (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Instalação, configuração e comissionamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mão de obra — passagem de cabos, fixação, configuração de VLANs/SSIDs, testes</t>
-  </si>
-  <si>
     <t xml:space="preserve">vb</t>
   </si>
   <si>
@@ -413,9 +344,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sem equipamentos elétricos na borda molhada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Garagem</t>
   </si>
   <si>
     <t xml:space="preserve">AP-04 (opcional, externo)</t>
@@ -590,14 +518,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFEDEDED"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
     <fill>
@@ -777,7 +705,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -797,6 +725,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -805,14 +741,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -825,7 +753,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1109,7 +1037,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1256,7 +1184,7 @@
         <v/>
       </c>
       <c r="J7" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1267,13 +1195,13 @@
         <v>13</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>1</v>
@@ -1287,7 +1215,7 @@
         <v/>
       </c>
       <c r="J8" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1298,13 +1226,13 @@
         <v>13</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>1</v>
@@ -1318,38 +1246,38 @@
         <v/>
       </c>
       <c r="J9" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="6" t="s">
+      <c r="B10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="C10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="4" t="s">
+      <c r="D10" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="8" t="str">
+      <c r="H10" s="12"/>
+      <c r="I10" s="13" t="str">
         <f aca="false">IF(H10="","",F10*H10)</f>
         <v/>
       </c>
-      <c r="J10" s="6" t="s">
-        <v>29</v>
+      <c r="J10" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1357,16 +1285,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>4</v>
@@ -1380,7 +1308,7 @@
         <v/>
       </c>
       <c r="J11" s="11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1388,19 +1316,19 @@
         <v>7</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>17</v>
@@ -1411,7 +1339,7 @@
         <v/>
       </c>
       <c r="J12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1419,19 +1347,19 @@
         <v>8</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>17</v>
@@ -1442,92 +1370,92 @@
         <v/>
       </c>
       <c r="J13" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="9" t="n">
+      <c r="B14" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="12"/>
-      <c r="I14" s="13" t="str">
+      <c r="G14" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="H14" s="17"/>
+      <c r="I14" s="18" t="str">
         <f aca="false">IF(H14="","",F14*H14)</f>
         <v/>
       </c>
-      <c r="J14" s="11" t="s">
+      <c r="J14" s="16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G15" s="9" t="s">
+      <c r="C15" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="12"/>
-      <c r="I15" s="13" t="str">
+      <c r="H15" s="17"/>
+      <c r="I15" s="18" t="str">
         <f aca="false">IF(H15="","",F15*H15)</f>
         <v/>
       </c>
-      <c r="J15" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J15" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="n">
         <v>11</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="H16" s="17"/>
       <c r="I16" s="18" t="str">
@@ -1538,444 +1466,165 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="n">
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="15" t="s">
+      <c r="B17" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="C17" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="D17" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="F17" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H17" s="17"/>
-      <c r="I17" s="18" t="str">
+      <c r="E17" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="H17" s="22"/>
+      <c r="I17" s="23" t="str">
         <f aca="false">IF(H17="","",F17*H17)</f>
         <v/>
       </c>
-      <c r="J17" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="n">
+      <c r="J17" s="21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="16" t="s">
+      <c r="B18" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="17"/>
-      <c r="I18" s="18" t="str">
+      <c r="D18" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="H18" s="22"/>
+      <c r="I18" s="23" t="str">
         <f aca="false">IF(H18="","",F18*H18)</f>
         <v/>
       </c>
-      <c r="J18" s="16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="n">
+      <c r="J18" s="21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E19" s="16" t="s">
+      <c r="B19" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H19" s="17"/>
-      <c r="I19" s="18" t="str">
+      <c r="D19" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="22"/>
+      <c r="I19" s="23" t="str">
         <f aca="false">IF(H19="","",F19*H19)</f>
         <v/>
       </c>
-      <c r="J19" s="16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="n">
+      <c r="J19" s="21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" s="16" t="s">
+      <c r="B20" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="F20" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="G20" s="14" t="s">
+      <c r="C20" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="H20" s="17"/>
-      <c r="I20" s="18" t="str">
+      <c r="D20" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="H20" s="27"/>
+      <c r="I20" s="28" t="str">
         <f aca="false">IF(H20="","",F20*H20)</f>
         <v/>
       </c>
-      <c r="J20" s="16" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="16" t="s">
+      <c r="J20" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="17"/>
-      <c r="I21" s="18" t="str">
-        <f aca="false">IF(H21="","",F21*H21)</f>
-        <v/>
-      </c>
-      <c r="J21" s="16" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30" t="n">
+        <f aca="false">SUM(I6:I20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E22" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H22" s="17"/>
-      <c r="I22" s="18" t="str">
-        <f aca="false">IF(H22="","",F22*H22)</f>
-        <v/>
-      </c>
-      <c r="J22" s="16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="F23" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H23" s="22"/>
-      <c r="I23" s="23" t="str">
-        <f aca="false">IF(H23="","",F23*H23)</f>
-        <v/>
-      </c>
-      <c r="J23" s="21" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="F24" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H24" s="22"/>
-      <c r="I24" s="23" t="str">
-        <f aca="false">IF(H24="","",F24*H24)</f>
-        <v/>
-      </c>
-      <c r="J24" s="21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23" t="str">
-        <f aca="false">IF(H25="","",F25*H25)</f>
-        <v/>
-      </c>
-      <c r="J25" s="21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C26" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="E26" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="F26" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H26" s="22"/>
-      <c r="I26" s="23" t="str">
-        <f aca="false">IF(H26="","",F26*H26)</f>
-        <v/>
-      </c>
-      <c r="J26" s="21" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="n">
-        <v>22</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="F27" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27" s="22"/>
-      <c r="I27" s="23" t="str">
-        <f aca="false">IF(H27="","",F27*H27)</f>
-        <v/>
-      </c>
-      <c r="J27" s="21" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="F28" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="22"/>
-      <c r="I28" s="23" t="str">
-        <f aca="false">IF(H28="","",F28*H28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="24" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="C29" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="E29" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="F29" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="H29" s="27"/>
-      <c r="I29" s="28" t="str">
-        <f aca="false">IF(H29="","",F29*H29)</f>
-        <v/>
-      </c>
-      <c r="J29" s="26" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29"/>
-      <c r="I31" s="30" t="n">
-        <f aca="false">SUM(I6:I29)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="C31:H31"/>
-    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="A24:J24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2001,7 +1650,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2011,10 +1660,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2022,69 +1671,69 @@
         <v>13</v>
       </c>
       <c r="B4" s="31" t="n">
-        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$29,A4)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$20,A4)</f>
+        <v>4</v>
       </c>
       <c r="C4" s="32" t="n">
-        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$29,A4,'Lista de Materiais'!$I$6:$I$29)</f>
+        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$20,A4,'Lista de Materiais'!$I$6:$I$20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B5" s="33" t="n">
-        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$29,A5)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$20,A5)</f>
+        <v>4</v>
       </c>
       <c r="C5" s="34" t="n">
-        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$29,A5,'Lista de Materiais'!$I$6:$I$29)</f>
+        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$20,A5,'Lista de Materiais'!$I$6:$I$20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B6" s="35" t="n">
-        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$29,A6)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$20,A6)</f>
+        <v>3</v>
       </c>
       <c r="C6" s="36" t="n">
-        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$29,A6,'Lista de Materiais'!$I$6:$I$29)</f>
+        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$20,A6,'Lista de Materiais'!$I$6:$I$20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="B7" s="37" t="n">
-        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$29,A7)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$20,A7)</f>
+        <v>3</v>
       </c>
       <c r="C7" s="38" t="n">
-        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$29,A7,'Lista de Materiais'!$I$6:$I$29)</f>
+        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$20,A7,'Lista de Materiais'!$I$6:$I$20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="39" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="B8" s="39" t="n">
-        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$29,A8)</f>
+        <f aca="false">COUNTIF('Lista de Materiais'!$B$6:$B$20,A8)</f>
         <v>1</v>
       </c>
       <c r="C8" s="40" t="n">
-        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$29,A8,'Lista de Materiais'!$I$6:$I$29)</f>
+        <f aca="false">SUMIF('Lista de Materiais'!$B$6:$B$20,A8,'Lista de Materiais'!$I$6:$I$20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="41" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="C10" s="42" t="n">
         <f aca="false">SUM(C4:C8)</f>
@@ -2120,7 +1769,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2129,7 +1778,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2138,189 +1787,189 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D5" s="43" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="B6" s="43" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D6" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="E6" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="D7" s="43" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="43" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="B8" s="43" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="D8" s="43" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="B9" s="43" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="D9" s="43" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="B10" s="43" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="D10" s="43" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E10" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="B11" s="43" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="D11" s="43" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="B12" s="43" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="D12" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="43" t="s">
-        <v>130</v>
+        <v>25</v>
       </c>
       <c r="B13" s="43" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="D13" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>133</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
-        <v>134</v>
+        <v>110</v>
       </c>
       <c r="B14" s="43" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="D14" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2354,7 +2003,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2362,7 +2011,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2370,59 +2019,59 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="44" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="B5" s="46" t="n">
         <v>165</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="D5" s="43" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>144</v>
+        <v>120</v>
       </c>
       <c r="B6" s="46" t="n">
         <v>7</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="D6" s="43" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
       <c r="B7" s="47" t="n">
         <f aca="false">(B5+B6)*0.15</f>
         <v>25.8</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="D7" s="43" t="s">
-        <v>147</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2433,30 +2082,30 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="48" t="s">
-        <v>148</v>
+        <v>124</v>
       </c>
       <c r="B9" s="49" t="n">
         <f aca="false">B5+B6+B7</f>
         <v>197.8</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="D9" s="43"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="B10" s="47" t="n">
         <f aca="false">ROUNDUP(B9/305,0)</f>
         <v>1</v>
       </c>
       <c r="C10" s="47" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D10" s="43" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Detalha metragem de cabo Cat6 por sistema e vincula ao rack unico
Aba Memoria de Calculo agora quebra a metragem de cabo por sistema em
vez de um total generico: Wi-Fi (4 pontos, 45m), CFTV (8 pontos, 80m),
TV (6 pontos, 60m) e uplink da ONU (10m), cada um ja com margem de
instalacao embutida. Total fecha em 195m, exigindo 1 caixa de 305m
com 110m de folga. A quantidade de caixas na Lista de Materiais agora
e uma formula que puxa direto dessa aba, eliminando qualquer risco de
os dois numeros ficarem incoerentes entre si.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fnpdJTGdpvo55JqsFcMfC
</commit_message>
<xml_diff>
--- a/SWISS-J26-Patrick/Lista_de_Materiais_Swiss_J26.xlsx
+++ b/SWISS-J26-Patrick/Lista_de_Materiais_Swiss_J26.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="131">
   <si>
     <t xml:space="preserve">Lista de Materiais — Rede Wi-Fi, CFTV e Cabeamento Estruturado</t>
   </si>
@@ -202,7 +202,7 @@
     <t xml:space="preserve">cx</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa ~198m (ver aba Memória de Cálculo) — 1 caixa cobre com folga</t>
+    <t xml:space="preserve">Atende os 18 pontos de rede (4 Wi-Fi + 8 CFTV + 6 TV) mais o uplink da ONU, já com margem de instalação — quantidade calculada na aba Memória de Cálculo</t>
   </si>
   <si>
     <t xml:space="preserve">Kit de terminação dos pontos de rede</t>
@@ -376,34 +376,46 @@
     <t xml:space="preserve">Unidade</t>
   </si>
   <si>
-    <t xml:space="preserve">Pontos internos/perimetrais (17 pontos: TVs+APs+câmeras) a partir do rack no Escritório</t>
+    <t xml:space="preserve">Wi-Fi — 4 pontos (AP-01, AP-02, AP-03 e AP-04 opcional)</t>
   </si>
   <si>
     <t xml:space="preserve">m</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa de escopo — item 6.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uplink ONU (Garagem) → rack (Escritório)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ponto médio da faixa 6-8m — item 6.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva de subida/descida, curvas e emendas (~15%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculada = (linha 5 + linha 6) x 15%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL ESTIMADO DE CABO CAT6</t>
+    <t xml:space="preserve">Distância-base ~39m + margem de instalação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CFTV — 8 pontos (CAM-01 a CAM-08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distância-base ~70m + margem de instalação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV — 6 pontos (Living, Suíte Master, Suíte 01, Suíte 02, Escritório, Gourmet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distância-base ~52m + margem de instalação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uplink ONU (Garagem) → Rack (Escritório)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distância-base ~6-8m + margem de instalação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL DE CABO CAT6 A COMPRAR</t>
   </si>
   <si>
     <t xml:space="preserve">Caixas de cabo Cat6 necessárias (305m cada)</t>
   </si>
   <si>
-    <t xml:space="preserve">Deve bater com a quantidade da Lista de Materiais</t>
+    <t xml:space="preserve">Puxado automaticamente para a Lista de Materiais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folga restante após atender todos os pontos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margem para ajustes de rota em campo</t>
   </si>
 </sst>
 </file>
@@ -1466,7 +1478,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="n">
         <v>12</v>
       </c>
@@ -1483,6 +1495,7 @@
         <v>57</v>
       </c>
       <c r="F17" s="19" t="n">
+        <f aca="false">'Memória de Cálculo'!B11</f>
         <v>1</v>
       </c>
       <c r="G17" s="19" t="s">
@@ -1992,13 +2005,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2031,12 +2044,12 @@
         <v>84</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
         <v>117</v>
       </c>
       <c r="B5" s="46" t="n">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="C5" s="47" t="s">
         <v>118</v>
@@ -2050,7 +2063,7 @@
         <v>120</v>
       </c>
       <c r="B6" s="46" t="n">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="C6" s="47" t="s">
         <v>118</v>
@@ -2063,9 +2076,8 @@
       <c r="A7" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="B7" s="47" t="n">
-        <f aca="false">(B5+B6)*0.15</f>
-        <v>25.8</v>
+      <c r="B7" s="46" t="n">
+        <v>60</v>
       </c>
       <c r="C7" s="47" t="s">
         <v>118</v>
@@ -2075,37 +2087,66 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="43"/>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="43"/>
+      <c r="A8" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="48" t="s">
-        <v>124</v>
-      </c>
-      <c r="B9" s="49" t="n">
-        <f aca="false">B5+B6+B7</f>
-        <v>197.8</v>
-      </c>
-      <c r="C9" s="47" t="s">
+      <c r="A9" s="43"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="43"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="48" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="49" t="n">
+        <f aca="false">SUM(B5:B8)</f>
+        <v>195</v>
+      </c>
+      <c r="C10" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="D9" s="43"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="43" t="s">
-        <v>125</v>
-      </c>
-      <c r="B10" s="47" t="n">
-        <f aca="false">ROUNDUP(B9/305,0)</f>
+      <c r="D10" s="43"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="48" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="49" t="n">
+        <f aca="false">ROUNDUP(B10/305,0)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="47" t="s">
+      <c r="C11" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="43" t="s">
-        <v>126</v>
+      <c r="D11" s="43" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="43" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" s="47" t="n">
+        <f aca="false">B11*305-B10</f>
+        <v>110</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>